<commit_message>
feat: establish full documentation for 2026 OBE curriculum implementation across multiple formats
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
+++ b/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
@@ -2725,12 +2725,12 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>`FST-409`</t>
+          <t>`STI-403`</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Manajemen Sains &amp; Riset Op</t>
+          <t>Pengantar NLP &amp; IR</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
@@ -2739,22 +2739,22 @@
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr"/>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>**R**</t>
-        </is>
-      </c>
+      <c r="F49" s="8" t="inlineStr"/>
       <c r="G49" s="8" t="inlineStr"/>
       <c r="H49" s="8" t="inlineStr"/>
-      <c r="I49" s="8" t="inlineStr">
+      <c r="I49" s="8" t="inlineStr"/>
+      <c r="J49" s="8" t="inlineStr">
         <is>
           <t>**R**</t>
         </is>
       </c>
-      <c r="J49" s="8" t="inlineStr"/>
       <c r="K49" s="8" t="inlineStr"/>
       <c r="L49" s="8" t="inlineStr"/>
-      <c r="M49" s="8" t="inlineStr"/>
+      <c r="M49" s="8" t="inlineStr">
+        <is>
+          <t>**R**</t>
+        </is>
+      </c>
       <c r="N49" s="8" t="inlineStr"/>
       <c r="O49" s="8" t="inlineStr"/>
       <c r="P49" s="8" t="inlineStr"/>
@@ -2762,12 +2762,12 @@
       <c r="R49" s="8" t="inlineStr"/>
       <c r="S49" s="8" t="inlineStr">
         <is>
-          <t>PL-1, PL-4</t>
+          <t>PL-1</t>
         </is>
       </c>
       <c r="T49" s="8" t="inlineStr">
         <is>
-          <t>PEO-1, PEO-2</t>
+          <t>PEO-1, PEO-3</t>
         </is>
       </c>
       <c r="U49" s="8" t="inlineStr">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t>`STI-102`, `STI-103`, `STI-201`, `STI-202`, `FST-408`, `FST-409`</t>
+          <t>`STI-102`, `STI-103`, `STI-201`, `STI-202`, `FST-408`</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
@@ -6482,7 +6482,7 @@
       </c>
       <c r="E137" s="8" t="inlineStr">
         <is>
-          <t>7 MK</t>
+          <t>6 MK</t>
         </is>
       </c>
       <c r="F137" s="8" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t>`STI-302`, `STI-601`, `STA-03`, `STA-05`</t>
+          <t>`STI-302`, `STI-403`, `STI-601`, `STA-03`, `STA-05`</t>
         </is>
       </c>
       <c r="D143" s="8" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="E143" s="8" t="inlineStr">
         <is>
-          <t>6 MK</t>
+          <t>7 MK</t>
         </is>
       </c>
       <c r="F143" s="8" t="inlineStr">
@@ -6869,7 +6869,7 @@
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t>`STI-302`, `STI-401`, `STI-501`, `STI-601`</t>
+          <t>`STI-302`, `STI-401`, `STI-403`, `STI-501`, `STI-601`</t>
         </is>
       </c>
       <c r="D151" s="8" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="E151" s="8" t="inlineStr">
         <is>
-          <t>8 MK</t>
+          <t>9 MK</t>
         </is>
       </c>
       <c r="F151" s="8" t="inlineStr">
@@ -8706,12 +8706,12 @@
       </c>
       <c r="B196" s="8" t="inlineStr">
         <is>
-          <t>`FST-409`</t>
+          <t>`STI-403`</t>
         </is>
       </c>
       <c r="C196" s="8" t="inlineStr">
         <is>
-          <t>Manajemen Sains &amp; Riset Op</t>
+          <t>Pengantar NLP &amp; IR</t>
         </is>
       </c>
       <c r="D196" s="10" t="inlineStr">
@@ -8721,22 +8721,22 @@
       </c>
       <c r="E196" s="8" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="F196" s="8" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="H196" s="8" t="inlineStr">
         <is>
-          <t>**50%**</t>
+          <t>**65%**</t>
         </is>
       </c>
       <c r="I196" s="8" t="inlineStr">

</xml_diff>

<commit_message>
refactor: swap Deep Learning to Sem 6 (STI-626) and Keamanan Informasi Lanjut to Sem 5 (STI-519)
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
+++ b/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>`STI-201`</t>
+          <t>`STI-204`</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>`STI-202`</t>
+          <t>`STI-205`</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>`STI-301`</t>
+          <t>`STI-306`</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>`STI-302`</t>
+          <t>`STI-307`</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>`STI-303`</t>
+          <t>`STI-308`</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>`STI-304`</t>
+          <t>`STI-309`</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>`STI-305`</t>
+          <t>`STI-310`</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>`STI-306`</t>
+          <t>`STI-311`</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>`STI-307`</t>
+          <t>`STI-312`</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>`STI-401`</t>
+          <t>`STI-413`</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>`STI-402`</t>
+          <t>`STI-415`</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>`STI-407`</t>
+          <t>`STI-416`</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>`STI-404`</t>
+          <t>`STI-417`</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>`STI-405`</t>
+          <t>`STI-418`</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>`STI-403`</t>
+          <t>`STI-414`</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -3037,12 +3037,12 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>`STI-501`</t>
+          <t>`STI-519`</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Deep Learning &amp; Neural Net</t>
+          <t>Keamanan Informasi Lanjut</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -3056,35 +3056,39 @@
       <c r="H55" s="7" t="inlineStr"/>
       <c r="I55" s="7" t="inlineStr"/>
       <c r="J55" s="7" t="inlineStr"/>
-      <c r="K55" s="7" t="inlineStr"/>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>**M**</t>
+        </is>
+      </c>
       <c r="L55" s="7" t="inlineStr"/>
-      <c r="M55" s="7" t="inlineStr">
-        <is>
-          <t>**R**</t>
-        </is>
-      </c>
-      <c r="N55" s="7" t="inlineStr">
-        <is>
-          <t>**R**</t>
-        </is>
-      </c>
-      <c r="O55" s="7" t="inlineStr"/>
-      <c r="P55" s="7" t="inlineStr"/>
+      <c r="M55" s="7" t="inlineStr"/>
+      <c r="N55" s="7" t="inlineStr"/>
+      <c r="O55" s="7" t="inlineStr">
+        <is>
+          <t>**M**</t>
+        </is>
+      </c>
+      <c r="P55" s="7" t="inlineStr">
+        <is>
+          <t>**M**</t>
+        </is>
+      </c>
       <c r="Q55" s="7" t="inlineStr"/>
       <c r="R55" s="7" t="inlineStr"/>
       <c r="S55" s="7" t="inlineStr">
         <is>
-          <t>PL-1</t>
+          <t>PL-2</t>
         </is>
       </c>
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>PEO-1, PEO-3</t>
+          <t>PEO-1</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
         <is>
-          <t>**R**</t>
+          <t>**M**</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3100,7 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>`STI-503`</t>
+          <t>`STI-520`</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
@@ -3155,7 +3159,7 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>`STI-504`</t>
+          <t>`STI-521`</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
@@ -3214,7 +3218,7 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>`STI-505`</t>
+          <t>`STI-522`</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -3273,7 +3277,7 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>`STI-506`</t>
+          <t>`STI-523`</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
@@ -3517,7 +3521,7 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>`STI-601`</t>
+          <t>`STI-624`</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -3576,7 +3580,7 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>`STI-602`</t>
+          <t>`STI-625`</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -3635,12 +3639,12 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>`STI-603`</t>
+          <t>`STI-626`</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Keamanan Informasi Lanjut</t>
+          <t>Deep Learning &amp; Neural Net</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3654,39 +3658,35 @@
       <c r="H65" s="7" t="inlineStr"/>
       <c r="I65" s="7" t="inlineStr"/>
       <c r="J65" s="7" t="inlineStr"/>
-      <c r="K65" s="7" t="inlineStr">
-        <is>
-          <t>**M**</t>
-        </is>
-      </c>
+      <c r="K65" s="7" t="inlineStr"/>
       <c r="L65" s="7" t="inlineStr"/>
-      <c r="M65" s="7" t="inlineStr"/>
-      <c r="N65" s="7" t="inlineStr"/>
-      <c r="O65" s="7" t="inlineStr">
-        <is>
-          <t>**M**</t>
-        </is>
-      </c>
-      <c r="P65" s="7" t="inlineStr">
-        <is>
-          <t>**M**</t>
-        </is>
-      </c>
+      <c r="M65" s="7" t="inlineStr">
+        <is>
+          <t>**R**</t>
+        </is>
+      </c>
+      <c r="N65" s="7" t="inlineStr">
+        <is>
+          <t>**R**</t>
+        </is>
+      </c>
+      <c r="O65" s="7" t="inlineStr"/>
+      <c r="P65" s="7" t="inlineStr"/>
       <c r="Q65" s="7" t="inlineStr"/>
       <c r="R65" s="7" t="inlineStr"/>
       <c r="S65" s="7" t="inlineStr">
         <is>
-          <t>PL-2</t>
+          <t>PL-1</t>
         </is>
       </c>
       <c r="T65" s="7" t="inlineStr">
         <is>
-          <t>PEO-1</t>
+          <t>PEO-1, PEO-3</t>
         </is>
       </c>
       <c r="U65" s="7" t="inlineStr">
         <is>
-          <t>**M**</t>
+          <t>**R**</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>`STI-604`</t>
+          <t>`STI-627`</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>`STI-701`</t>
+          <t>`STI-728`</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
@@ -6197,7 +6197,7 @@
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>`STI-301`</t>
+          <t>`STI-306`</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t>`FST-207`, `STI-402`, `STI-503`</t>
+          <t>`FST-207`, `STI-415`, `STI-520`</t>
         </is>
       </c>
       <c r="D129" s="8" t="inlineStr">
@@ -6256,12 +6256,12 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>`STI-103`, `STI-307`, `STI-404`, `STI-305`</t>
+          <t>`STI-103`, `STI-312`, `STI-417`, `STI-310`</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>`STB-01`, `STB-02`, `STI-504`</t>
+          <t>`STB-01`, `STB-02`, `STI-521`</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="D131" s="8" t="inlineStr">
         <is>
-          <t>`STI-301`, `STI-604`</t>
+          <t>`STI-306`, `STI-627`</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>`STI-506`, `STB-03`</t>
+          <t>`STI-523`, `STB-03`</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t>`STI-405`, `STI-603`, `STB-01`, `STB-03`</t>
+          <t>`STI-418`, `STI-519`, `STB-01`, `STB-03`</t>
         </is>
       </c>
       <c r="D133" s="8" t="inlineStr">
@@ -6384,7 +6384,7 @@
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>`STI-301`, `STI-304`</t>
+          <t>`STI-306`, `STI-309`</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t>`STI-506`, `STC-06`</t>
+          <t>`STI-523`, `STC-06`</t>
         </is>
       </c>
       <c r="D135" s="8" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>`STI-301`, `STI-602`</t>
+          <t>`STI-306`, `STI-625`</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t>`STI-102`, `STI-201`, `STI-202`, `FST-408`</t>
+          <t>`STI-102`, `STI-204`, `STI-205`, `FST-408`</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>`STI-306`, `STI-407`</t>
+          <t>`STI-311`, `STI-416`</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t>`STI-306`, `STI-407`, `STI-505`, `STI-604`</t>
+          <t>`STI-311`, `STI-416`, `STI-522`, `STI-627`</t>
         </is>
       </c>
       <c r="D139" s="8" t="inlineStr">
@@ -6576,12 +6576,12 @@
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>`STI-402`, `STI-503`, `STA-01`</t>
+          <t>`STI-415`, `STI-520`, `STA-01`</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>`STI-401`, `STA-04`</t>
+          <t>`STI-413`, `STA-04`</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>`MKU-204`, `STI-701`, `FST-610`</t>
+          <t>`MKU-204`, `STI-728`, `FST-610`</t>
         </is>
       </c>
       <c r="D142" s="9" t="inlineStr">
@@ -6672,12 +6672,12 @@
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t>`STI-302`, `STI-403`, `STI-601`, `STA-03`, `STA-05`</t>
+          <t>`STI-307`, `STI-414`, `STI-624`, `STA-03`, `STA-05`</t>
         </is>
       </c>
       <c r="D143" s="8" t="inlineStr">
         <is>
-          <t>`STI-401`, `STA-06`</t>
+          <t>`STI-413`, `STA-06`</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
@@ -6704,12 +6704,12 @@
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>`STI-303`, `STC-01`</t>
+          <t>`STI-308`, `STC-01`</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>`STI-306`, `STI-505`</t>
+          <t>`STI-311`, `STI-522`</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t>`STI-401`, `STI-501`, `STA-04`</t>
+          <t>`STI-413`, `STI-626`, `STA-04`</t>
         </is>
       </c>
       <c r="D145" s="8" t="inlineStr">
@@ -6768,12 +6768,12 @@
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>`STI-404`, `STB-02`</t>
+          <t>`STI-417`, `STB-02`</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>`STI-604`, `STC-05`</t>
+          <t>`STI-627`, `STC-05`</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="D147" s="8" t="inlineStr">
         <is>
-          <t>`STI-405`, `STI-602`, `STB-04`</t>
+          <t>`STI-418`, `STI-625`, `STB-04`</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -6941,7 +6941,7 @@
       </c>
       <c r="C153" s="8" t="inlineStr">
         <is>
-          <t>`STI-302`, `STI-401`, `STI-403`, `STI-501`, `STI-601`</t>
+          <t>`STI-307`, `STI-413`, `STI-414`, `STI-626`, `STI-624`</t>
         </is>
       </c>
       <c r="D153" s="8" t="inlineStr">
@@ -6973,12 +6973,12 @@
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>`STI-307`</t>
+          <t>`STI-312`</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>`STI-404`, `STI-504`, `STB-01`</t>
+          <t>`STI-417`, `STI-521`, `STB-01`</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="C155" s="8" t="inlineStr">
         <is>
-          <t>`STI-306`, `STI-407`, `STI-505`, `STI-604`</t>
+          <t>`STI-311`, `STI-416`, `STI-522`, `STI-627`</t>
         </is>
       </c>
       <c r="D155" s="8" t="inlineStr">
@@ -7037,12 +7037,12 @@
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>`STI-404`, `STB-02`</t>
+          <t>`STI-417`, `STB-02`</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>`STI-305`, `STC-05`</t>
+          <t>`STI-310`, `STC-05`</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
@@ -7069,7 +7069,7 @@
       </c>
       <c r="C157" s="8" t="inlineStr">
         <is>
-          <t>`STI-405`, `STI-603`, `STB-01`</t>
+          <t>`STI-418`, `STI-519`, `STB-01`</t>
         </is>
       </c>
       <c r="D157" s="10" t="inlineStr">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>`STI-601`, `STI-604`, `FST-610`</t>
+          <t>`STI-624`, `STI-627`, `FST-610`</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="D159" s="8" t="inlineStr">
         <is>
-          <t>`STI-506`</t>
+          <t>`STI-523`</t>
         </is>
       </c>
       <c r="E159" s="8" t="inlineStr">
@@ -7165,7 +7165,7 @@
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>`STI-402`, `STI-503`</t>
+          <t>`STI-415`, `STI-520`</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
@@ -7197,12 +7197,12 @@
       </c>
       <c r="C161" s="8" t="inlineStr">
         <is>
-          <t>`STI-303`, `STC-01`</t>
+          <t>`STI-308`, `STC-01`</t>
         </is>
       </c>
       <c r="D161" s="8" t="inlineStr">
         <is>
-          <t>`STI-306`, `STC-04`</t>
+          <t>`STI-311`, `STC-04`</t>
         </is>
       </c>
       <c r="E161" s="8" t="inlineStr">
@@ -7229,7 +7229,7 @@
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>`STI-304`, `STI-407`, `STI-604`</t>
+          <t>`STI-309`, `STI-416`, `STI-627`</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
@@ -7293,7 +7293,7 @@
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>`MKU-204`, `STI-701`, `FST-610`</t>
+          <t>`MKU-204`, `STI-728`, `FST-610`</t>
         </is>
       </c>
       <c r="D164" s="9" t="inlineStr">
@@ -7325,12 +7325,12 @@
       </c>
       <c r="C165" s="8" t="inlineStr">
         <is>
-          <t>`STI-504`, `STA-06`</t>
+          <t>`STI-521`, `STA-06`</t>
         </is>
       </c>
       <c r="D165" s="8" t="inlineStr">
         <is>
-          <t>`STI-305`, `STI-307`</t>
+          <t>`STI-310`, `STI-312`</t>
         </is>
       </c>
       <c r="E165" s="8" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="B178" s="7" t="inlineStr">
         <is>
-          <t>`STI-201`</t>
+          <t>`STI-204`</t>
         </is>
       </c>
       <c r="C178" s="7" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="B179" s="8" t="inlineStr">
         <is>
-          <t>`STI-202`</t>
+          <t>`STI-205`</t>
         </is>
       </c>
       <c r="C179" s="8" t="inlineStr">
@@ -8199,7 +8199,7 @@
       </c>
       <c r="B186" s="7" t="inlineStr">
         <is>
-          <t>`STI-301`</t>
+          <t>`STI-306`</t>
         </is>
       </c>
       <c r="C186" s="7" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="B187" s="8" t="inlineStr">
         <is>
-          <t>`STI-302`</t>
+          <t>`STI-307`</t>
         </is>
       </c>
       <c r="C187" s="8" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="B188" s="7" t="inlineStr">
         <is>
-          <t>`STI-303`</t>
+          <t>`STI-308`</t>
         </is>
       </c>
       <c r="C188" s="7" t="inlineStr">
@@ -8340,7 +8340,7 @@
       </c>
       <c r="B189" s="8" t="inlineStr">
         <is>
-          <t>`STI-304`</t>
+          <t>`STI-309`</t>
         </is>
       </c>
       <c r="C189" s="8" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="B190" s="7" t="inlineStr">
         <is>
-          <t>`STI-305`</t>
+          <t>`STI-310`</t>
         </is>
       </c>
       <c r="C190" s="7" t="inlineStr">
@@ -8434,7 +8434,7 @@
       </c>
       <c r="B191" s="8" t="inlineStr">
         <is>
-          <t>`STI-306`</t>
+          <t>`STI-311`</t>
         </is>
       </c>
       <c r="C191" s="8" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="B192" s="7" t="inlineStr">
         <is>
-          <t>`STI-307`</t>
+          <t>`STI-312`</t>
         </is>
       </c>
       <c r="C192" s="7" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="B193" s="8" t="inlineStr">
         <is>
-          <t>`STI-401`</t>
+          <t>`STI-413`</t>
         </is>
       </c>
       <c r="C193" s="8" t="inlineStr">
@@ -8575,7 +8575,7 @@
       </c>
       <c r="B194" s="7" t="inlineStr">
         <is>
-          <t>`STI-402`</t>
+          <t>`STI-415`</t>
         </is>
       </c>
       <c r="C194" s="7" t="inlineStr">
@@ -8622,7 +8622,7 @@
       </c>
       <c r="B195" s="8" t="inlineStr">
         <is>
-          <t>`STI-407`</t>
+          <t>`STI-416`</t>
         </is>
       </c>
       <c r="C195" s="8" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="B196" s="7" t="inlineStr">
         <is>
-          <t>`STI-404`</t>
+          <t>`STI-417`</t>
         </is>
       </c>
       <c r="C196" s="7" t="inlineStr">
@@ -8716,7 +8716,7 @@
       </c>
       <c r="B197" s="8" t="inlineStr">
         <is>
-          <t>`STI-405`</t>
+          <t>`STI-418`</t>
         </is>
       </c>
       <c r="C197" s="8" t="inlineStr">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="B199" s="8" t="inlineStr">
         <is>
-          <t>`STI-403`</t>
+          <t>`STI-414`</t>
         </is>
       </c>
       <c r="C199" s="8" t="inlineStr">
@@ -8904,12 +8904,12 @@
       </c>
       <c r="B201" s="8" t="inlineStr">
         <is>
-          <t>`STI-501`</t>
+          <t>`STI-519`</t>
         </is>
       </c>
       <c r="C201" s="8" t="inlineStr">
         <is>
-          <t>Deep Learning &amp; Neural Net</t>
+          <t>Keamanan Informasi Lanjut</t>
         </is>
       </c>
       <c r="D201" s="10" t="inlineStr">
@@ -8919,12 +8919,12 @@
       </c>
       <c r="E201" s="8" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="F201" s="8" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="G201" s="8" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="B202" s="7" t="inlineStr">
         <is>
-          <t>`STI-503`</t>
+          <t>`STI-520`</t>
         </is>
       </c>
       <c r="C202" s="7" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="B203" s="8" t="inlineStr">
         <is>
-          <t>`STI-504`</t>
+          <t>`STI-521`</t>
         </is>
       </c>
       <c r="C203" s="8" t="inlineStr">
@@ -9045,7 +9045,7 @@
       </c>
       <c r="B204" s="7" t="inlineStr">
         <is>
-          <t>`STI-505`</t>
+          <t>`STI-522`</t>
         </is>
       </c>
       <c r="C204" s="7" t="inlineStr">
@@ -9092,7 +9092,7 @@
       </c>
       <c r="B205" s="8" t="inlineStr">
         <is>
-          <t>`STI-506`</t>
+          <t>`STI-523`</t>
         </is>
       </c>
       <c r="C205" s="8" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="B209" s="8" t="inlineStr">
         <is>
-          <t>`STI-601`</t>
+          <t>`STI-624`</t>
         </is>
       </c>
       <c r="C209" s="8" t="inlineStr">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="B210" s="7" t="inlineStr">
         <is>
-          <t>`STI-602`</t>
+          <t>`STI-625`</t>
         </is>
       </c>
       <c r="C210" s="7" t="inlineStr">
@@ -9374,12 +9374,12 @@
       </c>
       <c r="B211" s="8" t="inlineStr">
         <is>
-          <t>`STI-603`</t>
+          <t>`STI-626`</t>
         </is>
       </c>
       <c r="C211" s="8" t="inlineStr">
         <is>
-          <t>Keamanan Informasi Lanjut</t>
+          <t>Deep Learning &amp; Neural Net</t>
         </is>
       </c>
       <c r="D211" s="10" t="inlineStr">
@@ -9389,12 +9389,12 @@
       </c>
       <c r="E211" s="8" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="F211" s="8" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G211" s="8" t="inlineStr">
@@ -9421,7 +9421,7 @@
       </c>
       <c r="B212" s="7" t="inlineStr">
         <is>
-          <t>`STI-604`</t>
+          <t>`STI-627`</t>
         </is>
       </c>
       <c r="C212" s="7" t="inlineStr">
@@ -9609,7 +9609,7 @@
       </c>
       <c r="B216" s="7" t="inlineStr">
         <is>
-          <t>`STI-701`</t>
+          <t>`STI-728`</t>
         </is>
       </c>
       <c r="C216" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat: initialize curriculum 2026 revision documentation suite and supporting automation tools
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
+++ b/KURIKULUM2026_REVISI/004_MATRIKS_KETERLACAKAN_OBE_VMTS_PEO_PL_CPL_MK.xlsx
@@ -4790,9 +4790,9 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B84" s="9" t="inlineStr">
-        <is>
-          <t>`STA-01`</t>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>`STA-501`</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
@@ -4837,9 +4837,9 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B85" s="10" t="inlineStr">
-        <is>
-          <t>`STA-02`</t>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>`STA-601`</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
@@ -4884,9 +4884,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B86" s="9" t="inlineStr">
-        <is>
-          <t>`STA-03`</t>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>`STA-602`</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
@@ -4931,9 +4931,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B87" s="10" t="inlineStr">
-        <is>
-          <t>`STA-04`</t>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>`STA-701`</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
@@ -4978,9 +4978,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B88" s="9" t="inlineStr">
-        <is>
-          <t>`STA-05`</t>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>`STA-702`</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
@@ -5025,9 +5025,9 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B89" s="10" t="inlineStr">
-        <is>
-          <t>`STA-06`</t>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>`STA-703`</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
@@ -5135,9 +5135,9 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B93" s="9" t="inlineStr">
-        <is>
-          <t>`STB-01`</t>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>`STB-501`</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
@@ -5182,9 +5182,9 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B94" s="10" t="inlineStr">
-        <is>
-          <t>`STB-02`</t>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>`STB-601`</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
@@ -5229,9 +5229,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B95" s="9" t="inlineStr">
-        <is>
-          <t>`STB-03`</t>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>`STB-602`</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
@@ -5276,9 +5276,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B96" s="10" t="inlineStr">
-        <is>
-          <t>`STB-04`</t>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>`STB-701`</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
@@ -5323,9 +5323,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B97" s="9" t="inlineStr">
-        <is>
-          <t>`STB-05`</t>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>`STB-702`</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -5370,9 +5370,9 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B98" s="10" t="inlineStr">
-        <is>
-          <t>`STB-06`</t>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>`STB-703`</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
@@ -5480,9 +5480,9 @@
           <t>1</t>
         </is>
       </c>
-      <c r="B102" s="9" t="inlineStr">
-        <is>
-          <t>`STC-01`</t>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t>`STC-501`</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
@@ -5527,9 +5527,9 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B103" s="10" t="inlineStr">
-        <is>
-          <t>`STC-02`</t>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>`STC-601`</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
@@ -5574,9 +5574,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B104" s="9" t="inlineStr">
-        <is>
-          <t>`STC-03`</t>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>`STC-602`</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
@@ -5621,9 +5621,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B105" s="10" t="inlineStr">
-        <is>
-          <t>`STC-04`</t>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>`STC-701`</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
@@ -5668,9 +5668,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B106" s="9" t="inlineStr">
-        <is>
-          <t>`STC-05`</t>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>`STC-702`</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
@@ -5715,9 +5715,9 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B107" s="10" t="inlineStr">
-        <is>
-          <t>`STC-06`</t>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>`STC-703`</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
@@ -6229,7 +6229,7 @@
       </c>
       <c r="D129" s="8" t="inlineStr">
         <is>
-          <t>`STA-01`, `STA-04`</t>
+          <t>`STA-501`, `STA-701`</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
@@ -6261,7 +6261,7 @@
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>`STB-01`, `STB-02`, `STI-521`</t>
+          <t>`STB-501`, `STB-601`, `STI-521`</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
@@ -6286,9 +6286,9 @@
           <t>*Enterprise Architecture*</t>
         </is>
       </c>
-      <c r="C131" s="10" t="inlineStr">
-        <is>
-          <t>`STB-06`</t>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>`STB-703`</t>
         </is>
       </c>
       <c r="D131" s="8" t="inlineStr">
@@ -6320,12 +6320,12 @@
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>`STB-04`, `STB-05`</t>
+          <t>`STB-701`, `STB-702`</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>`STI-523`, `STB-03`</t>
+          <t>`STI-523`, `STB-602`</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t>`STI-418`, `STI-519`, `STB-01`, `STB-03`</t>
+          <t>`STI-418`, `STI-519`, `STB-501`, `STB-602`</t>
         </is>
       </c>
       <c r="D133" s="8" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>`FST-610`, `STC-02`</t>
+          <t>`FST-610`, `STC-601`</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t>`STI-523`, `STC-06`</t>
+          <t>`STI-523`, `STC-703`</t>
         </is>
       </c>
       <c r="D135" s="8" t="inlineStr">
@@ -6446,9 +6446,9 @@
           <t>*Business Process Management*</t>
         </is>
       </c>
-      <c r="C136" s="9" t="inlineStr">
-        <is>
-          <t>`STC-02`</t>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
+          <t>`STC-601`</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
@@ -6483,9 +6483,9 @@
           <t>`STI-102`, `STI-204`, `STI-205`, `FST-408`</t>
         </is>
       </c>
-      <c r="D137" s="10" t="inlineStr">
-        <is>
-          <t>`STA-02`</t>
+      <c r="D137" s="8" t="inlineStr">
+        <is>
+          <t>`STA-601`</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
@@ -6549,7 +6549,7 @@
       </c>
       <c r="D139" s="8" t="inlineStr">
         <is>
-          <t>`STC-03`, `STC-05`</t>
+          <t>`STC-602`, `STC-702`</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -6576,12 +6576,12 @@
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>`STI-415`, `STI-520`, `STA-01`</t>
+          <t>`STI-415`, `STI-520`, `STA-501`</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>`STI-413`, `STA-04`</t>
+          <t>`STI-413`, `STA-701`</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
@@ -6608,12 +6608,12 @@
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t>`STB-04`, `STB-03`</t>
+          <t>`STB-701`, `STB-602`</t>
         </is>
       </c>
       <c r="D141" s="8" t="inlineStr">
         <is>
-          <t>`FST-206`, `STB-05`</t>
+          <t>`FST-206`, `STB-702`</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -6643,9 +6643,9 @@
           <t>`MKU-204`, `STI-728`, `FST-610`</t>
         </is>
       </c>
-      <c r="D142" s="9" t="inlineStr">
-        <is>
-          <t>`STC-06`</t>
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t>`STC-703`</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
@@ -6672,12 +6672,12 @@
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t>`STI-307`, `STI-414`, `STI-624`, `STA-03`, `STA-05`</t>
+          <t>`STI-307`, `STI-414`, `STI-624`, `STA-602`, `STA-702`</t>
         </is>
       </c>
       <c r="D143" s="8" t="inlineStr">
         <is>
-          <t>`STI-413`, `STA-06`</t>
+          <t>`STI-413`, `STA-703`</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>`STI-308`, `STC-01`</t>
+          <t>`STI-308`, `STC-501`</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
@@ -6736,12 +6736,12 @@
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t>`STI-413`, `STI-626`, `STA-04`</t>
+          <t>`STI-413`, `STI-626`, `STA-701`</t>
         </is>
       </c>
       <c r="D145" s="8" t="inlineStr">
         <is>
-          <t>`STA-02`, `STA-06`</t>
+          <t>`STA-601`, `STA-703`</t>
         </is>
       </c>
       <c r="E145" s="8" t="inlineStr">
@@ -6768,12 +6768,12 @@
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>`STI-417`, `STB-02`</t>
+          <t>`STI-417`, `STB-601`</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>`STI-627`, `STC-05`</t>
+          <t>`STI-627`, `STC-702`</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="D147" s="8" t="inlineStr">
         <is>
-          <t>`STI-418`, `STI-625`, `STB-04`</t>
+          <t>`STI-418`, `STI-625`, `STB-701`</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="D153" s="8" t="inlineStr">
         <is>
-          <t>`STA-03..06`</t>
+          <t>`STA-602, STA-701..703`</t>
         </is>
       </c>
       <c r="E153" s="8" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>`STI-417`, `STI-521`, `STB-01`</t>
+          <t>`STI-417`, `STI-521`, `STB-501`</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="D155" s="8" t="inlineStr">
         <is>
-          <t>`STC-03..05`</t>
+          <t>`STC-602, STC-701..702`</t>
         </is>
       </c>
       <c r="E155" s="8" t="inlineStr">
@@ -7037,12 +7037,12 @@
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>`STI-417`, `STB-02`</t>
+          <t>`STI-417`, `STB-601`</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>`STI-310`, `STC-05`</t>
+          <t>`STI-310`, `STC-702`</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
@@ -7069,12 +7069,12 @@
       </c>
       <c r="C157" s="8" t="inlineStr">
         <is>
-          <t>`STI-418`, `STI-519`, `STB-01`</t>
-        </is>
-      </c>
-      <c r="D157" s="10" t="inlineStr">
-        <is>
-          <t>`STB-03`</t>
+          <t>`STI-418`, `STI-519`, `STB-501`</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="inlineStr">
+        <is>
+          <t>`STB-602`</t>
         </is>
       </c>
       <c r="E157" s="8" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>`STB-06`, `STC-02`</t>
+          <t>`STB-703`, `STC-601`</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
@@ -7133,7 +7133,7 @@
       </c>
       <c r="C159" s="8" t="inlineStr">
         <is>
-          <t>`STB-04`, `STB-05`</t>
+          <t>`STB-701`, `STB-702`</t>
         </is>
       </c>
       <c r="D159" s="8" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>`STA-01`, `STA-04`</t>
+          <t>`STA-501`, `STA-701`</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
@@ -7197,12 +7197,12 @@
       </c>
       <c r="C161" s="8" t="inlineStr">
         <is>
-          <t>`STI-308`, `STC-01`</t>
+          <t>`STI-308`, `STC-501`</t>
         </is>
       </c>
       <c r="D161" s="8" t="inlineStr">
         <is>
-          <t>`STI-311`, `STC-04`</t>
+          <t>`STI-311`, `STC-701`</t>
         </is>
       </c>
       <c r="E161" s="8" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>`FST-205`, `STC-05`</t>
+          <t>`FST-205`, `STC-702`</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
@@ -7261,7 +7261,7 @@
       </c>
       <c r="C163" s="8" t="inlineStr">
         <is>
-          <t>`STB-03`, `STB-04`</t>
+          <t>`STB-602`, `STB-701`</t>
         </is>
       </c>
       <c r="D163" s="8" t="inlineStr">
@@ -7296,9 +7296,9 @@
           <t>`MKU-204`, `STI-728`, `FST-610`</t>
         </is>
       </c>
-      <c r="D164" s="9" t="inlineStr">
-        <is>
-          <t>`STC-06`</t>
+      <c r="D164" s="7" t="inlineStr">
+        <is>
+          <t>`STC-703`</t>
         </is>
       </c>
       <c r="E164" s="7" t="inlineStr">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="C165" s="8" t="inlineStr">
         <is>
-          <t>`STI-521`, `STA-06`</t>
+          <t>`STI-521`, `STA-703`</t>
         </is>
       </c>
       <c r="D165" s="8" t="inlineStr">

</xml_diff>